<commit_message>
smol avance is still avance
</commit_message>
<xml_diff>
--- a/Shear Stress/stress_partitioning/cross_sectional_weirdness.xlsx
+++ b/Shear Stress/stress_partitioning/cross_sectional_weirdness.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huck4481\Documents\GitHub\La_Jara\Shear Stress\stress_partitioning\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicol\Documents\GitHub\La_Jara\Shear Stress\stress_partitioning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{98274C5F-ABCC-4106-A2B9-904D7AF1F5AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67A6A7DD-C4D6-41D5-8416-4A5946033A86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25320" yWindow="360" windowWidth="25440" windowHeight="15270" xr2:uid="{0C0685F1-586E-4A5C-BDE6-E93B881E3C00}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0C0685F1-586E-4A5C-BDE6-E93B881E3C00}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="14">
   <si>
     <t>ST2</t>
   </si>
@@ -66,12 +66,27 @@
   </si>
   <si>
     <t>all piezos</t>
+  </si>
+  <si>
+    <t>tau*</t>
+  </si>
+  <si>
+    <t>D50</t>
+  </si>
+  <si>
+    <t>mm</t>
+  </si>
+  <si>
+    <t>just p2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="167" formatCode="0.0000"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -101,8 +116,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -437,98 +458,211 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAF87FF3-2E1F-4937-B110-732DA535907A}">
-  <dimension ref="B1:E8"/>
+  <dimension ref="B1:K10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C1" t="s">
+    <row r="1" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
+      <c r="G1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D2">
+      <c r="C2" s="1"/>
+      <c r="D2" s="1">
         <v>8</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="1">
         <v>26</v>
       </c>
-    </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
+      <c r="G2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="I2" s="2">
+        <f>D2/((2650-1000)*9.81*$C$10/1000)</f>
+        <v>1.1232705144298138E-2</v>
+      </c>
+      <c r="J2" s="2">
+        <f>E2/((2650-1000)*9.81*$C$10/1000)</f>
+        <v>3.650629171896895E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D3">
+      <c r="C3" s="1"/>
+      <c r="D3" s="1">
         <v>10</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="1">
         <v>37</v>
       </c>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
+      <c r="G3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I3" s="2">
+        <f t="shared" ref="I3:J8" si="0">D3/((2650-1000)*9.81*$C$10/1000)</f>
+        <v>1.4040881430372673E-2</v>
+      </c>
+      <c r="J3" s="2">
+        <f t="shared" si="0"/>
+        <v>5.1951261292378891E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="1">
         <v>155</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="1">
         <v>40</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="1">
         <v>150</v>
       </c>
-    </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
+      <c r="G4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4" s="2">
+        <f t="shared" si="0"/>
+        <v>5.6163525721490692E-2</v>
+      </c>
+      <c r="J4" s="2">
+        <f t="shared" si="0"/>
+        <v>0.21061322145559008</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D5">
+      <c r="C5" s="1"/>
+      <c r="D5" s="1">
         <v>9.5</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="1">
         <v>25</v>
       </c>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B6" t="s">
+      <c r="G5" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="I5" s="2">
+        <f t="shared" si="0"/>
+        <v>1.3338837358854039E-2</v>
+      </c>
+      <c r="J5" s="2">
+        <f t="shared" si="0"/>
+        <v>3.5102203575931683E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D6">
+      <c r="C6" s="1"/>
+      <c r="D6" s="1">
         <v>4.3</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B7" t="s">
+      <c r="G6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="I6" s="2">
+        <f t="shared" si="0"/>
+        <v>6.0375790150602494E-3</v>
+      </c>
+      <c r="J6" s="2">
+        <f t="shared" si="0"/>
+        <v>4.2122644291118019E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D7">
+      <c r="C7" s="1"/>
+      <c r="D7" s="1">
         <v>4.2</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
+      <c r="G7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="I7" s="2">
+        <f t="shared" si="0"/>
+        <v>5.8971702007565227E-3</v>
+      </c>
+      <c r="J7" s="2">
+        <f t="shared" si="0"/>
+        <v>4.2122644291118019E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D8">
+      <c r="C8" s="1"/>
+      <c r="D8" s="1">
         <v>6</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="1">
         <v>7.9</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I8" s="2">
+        <f t="shared" si="0"/>
+        <v>8.4245288582236039E-3</v>
+      </c>
+      <c r="J8" s="2">
+        <f t="shared" si="0"/>
+        <v>1.1092296329994412E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B10" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10">
+        <v>44</v>
+      </c>
+      <c r="D10" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
shear stresses are correct! using p2 and p3
</commit_message>
<xml_diff>
--- a/Shear Stress/stress_partitioning/cross_sectional_weirdness.xlsx
+++ b/Shear Stress/stress_partitioning/cross_sectional_weirdness.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicol\Documents\GitHub\La_Jara\Shear Stress\stress_partitioning\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huck4481\Documents\GitHub\La_Jara\Shear Stress\stress_partitioning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67A6A7DD-C4D6-41D5-8416-4A5946033A86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D2976C2-FAB7-45D0-B36C-1095C2FA7BBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0C0685F1-586E-4A5C-BDE6-E93B881E3C00}"/>
+    <workbookView xWindow="-25320" yWindow="360" windowWidth="25440" windowHeight="15270" xr2:uid="{0C0685F1-586E-4A5C-BDE6-E93B881E3C00}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="13">
   <si>
     <t>ST2</t>
   </si>
@@ -75,9 +75,6 @@
   </si>
   <si>
     <t>mm</t>
-  </si>
-  <si>
-    <t>just p2</t>
   </si>
 </sst>
 </file>
@@ -85,7 +82,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="167" formatCode="0.0000"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -121,7 +118,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -487,9 +484,7 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="K1" s="1"/>
     </row>
     <row r="2" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">

</xml_diff>